<commit_message>
feat:improved empty names strategy
</commit_message>
<xml_diff>
--- a/data/output/authors_empty_names_elastic.xlsx
+++ b/data/output/authors_empty_names_elastic.xlsx
@@ -577,17 +577,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-02-03T07:57:25Z</t>
+          <t>2026-06-17T18:15:36Z</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>['ftniigatauniv:oai:niigata-u.repo.nii.ac.jp:00033599']</t>
+          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00027256']</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>['socio', 'edu']</t>
+          <t>['relig', 'litt']</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -601,7 +601,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>__-ovY2V8WJaJtQE9crlcID</t>
+          <t>__-lON76W5CSnNMbkPAYezr</t>
         </is>
       </c>
       <c r="H4" t="inlineStr"/>
@@ -625,17 +625,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-02-21T07:47:40Z</t>
+          <t>2026-08-14T13:09:35Z</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>['ftniigatauniv:oai:niigata-u.repo.nii.ac.jp:00007424']</t>
+          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00029930']</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>['scipo', 'envir']</t>
+          <t>['psy', 'lang']</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -649,7 +649,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>__-naeIh99PuU3iN80QFVuS</t>
+          <t>__-IaGDaXcYTDnsBd3RzrgY</t>
         </is>
       </c>
       <c r="H5" t="inlineStr"/>
@@ -673,17 +673,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-06-17T18:15:36Z</t>
+          <t>2026-02-03T07:57:25Z</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00027256']</t>
+          <t>['ftniigatauniv:oai:niigata-u.repo.nii.ac.jp:00033599']</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>['relig', 'litt']</t>
+          <t>['socio', 'edu']</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -697,7 +697,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>__-lON76W5CSnNMbkPAYezr</t>
+          <t>__-ovY2V8WJaJtQE9crlcID</t>
         </is>
       </c>
       <c r="H6" t="inlineStr"/>
@@ -721,17 +721,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-08-14T13:09:35Z</t>
+          <t>2026-02-21T07:47:40Z</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00029930']</t>
+          <t>['ftniigatauniv:oai:niigata-u.repo.nii.ac.jp:00007424']</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>['psy', 'lang']</t>
+          <t>['scipo', 'envir']</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -745,7 +745,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>__-IaGDaXcYTDnsBd3RzrgY</t>
+          <t>__-naeIh99PuU3iN80QFVuS</t>
         </is>
       </c>
       <c r="H7" t="inlineStr"/>
@@ -769,17 +769,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-02-03T07:57:29Z</t>
+          <t>2026-08-08T17:09:21Z</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>['ftniigatauniv:oai:niigata-u.repo.nii.ac.jp:00033599']</t>
+          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00016878']</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>['socio', 'edu']</t>
+          <t>['scipo', 'droit']</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -793,7 +793,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>__0T8inb4rnvx93h5vRc2Wz</t>
+          <t>__178mD65TgTNLB_U4mfAMi</t>
         </is>
       </c>
       <c r="H8" t="inlineStr"/>
@@ -817,17 +817,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-08-13T04:58:54Z</t>
+          <t>2026-08-13T04:58:51Z</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00026875']</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>['anthro-se', 'hist']</t>
+          <t>['relig', 'anthro-se']</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -841,12 +841,12 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>__1bKMVZRF2lGHXw5BAhc6F</t>
+          <t>__0gouguXks2rqD7ALw3QCU</t>
         </is>
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J9" t="b">
         <v>0</v>
@@ -865,17 +865,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-08-13T14:25:52Z</t>
+          <t>2026-02-03T07:57:29Z</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00027343']</t>
+          <t>['ftniigatauniv:oai:niigata-u.repo.nii.ac.jp:00033599']</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>['hisphilso', 'hist']</t>
+          <t>['socio', 'edu']</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -889,7 +889,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>__1RN_-bmxxkGhUlVjIxZF3</t>
+          <t>__0T8inb4rnvx93h5vRc2Wz</t>
         </is>
       </c>
       <c r="H10" t="inlineStr"/>
@@ -913,17 +913,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-08-13T04:58:51Z</t>
+          <t>2026-08-13T04:58:54Z</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00026875']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>['relig', 'anthro-se']</t>
+          <t>['anthro-se', 'hist']</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -937,12 +937,12 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>__0gouguXks2rqD7ALw3QCU</t>
+          <t>__1bKMVZRF2lGHXw5BAhc6F</t>
         </is>
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J11" t="b">
         <v>0</v>
@@ -1057,17 +1057,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-08-08T17:09:21Z</t>
+          <t>2026-08-13T14:25:52Z</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00016878']</t>
+          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00027343']</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>['scipo', 'droit']</t>
+          <t>['hisphilso', 'hist']</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1081,7 +1081,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>__178mD65TgTNLB_U4mfAMi</t>
+          <t>__1RN_-bmxxkGhUlVjIxZF3</t>
         </is>
       </c>
       <c r="H14" t="inlineStr"/>
@@ -1345,17 +1345,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-08-13T05:07:20Z</t>
+          <t>2026-08-10T07:04:30Z</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00029742']</t>
+          <t>['ftniigatauniv:oai:niigata-u.repo.nii.ac.jp:00007948']</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>['genre', 'socio']</t>
+          <t>['phil', 'edu']</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -1369,7 +1369,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>__3_t58xs1cQLEgcxtJJpog</t>
+          <t>__3_jse8IHzt0CU0dNALT6S</t>
         </is>
       </c>
       <c r="H20" t="inlineStr"/>
@@ -1393,17 +1393,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-02-20T08:04:15Z</t>
+          <t>2026-08-13T05:07:20Z</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>['ftniigatauniv:oai:niigata-u.repo.nii.ac.jp:00001726']</t>
+          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00029742']</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>['info', 'stat']</t>
+          <t>['genre', 'socio']</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -1417,7 +1417,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>__43texLZBHHfWpznk4gK0n</t>
+          <t>__3_t58xs1cQLEgcxtJJpog</t>
         </is>
       </c>
       <c r="H21" t="inlineStr"/>
@@ -1441,17 +1441,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-08-14T13:09:35Z</t>
+          <t>2026-02-20T08:04:15Z</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00029930']</t>
+          <t>['ftniigatauniv:oai:niigata-u.repo.nii.ac.jp:00001726']</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>['psy', 'lang']</t>
+          <t>['info', 'stat']</t>
         </is>
       </c>
       <c r="D22" t="n">
@@ -1465,7 +1465,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>__4ImgOXJRBqVTNim6hS9B9</t>
+          <t>__43texLZBHHfWpznk4gK0n</t>
         </is>
       </c>
       <c r="H22" t="inlineStr"/>
@@ -1489,17 +1489,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-08-10T07:04:30Z</t>
+          <t>2026-08-14T13:09:35Z</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>['ftniigatauniv:oai:niigata-u.repo.nii.ac.jp:00007948']</t>
+          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00029930']</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>['phil', 'edu']</t>
+          <t>['psy', 'lang']</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -1513,7 +1513,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>__3_jse8IHzt0CU0dNALT6S</t>
+          <t>__4ImgOXJRBqVTNim6hS9B9</t>
         </is>
       </c>
       <c r="H23" t="inlineStr"/>
@@ -1537,17 +1537,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-06-08T12:24:26Z</t>
+          <t>2026-08-14T11:54:29Z</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00025085']</t>
+          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00039136']</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>['museo']</t>
+          <t>['psy', 'lang']</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -1561,7 +1561,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>__4KN7H5ulJXhqUvCG7ZrPJ</t>
+          <t>__4eIpzAs05B4ZRv-5WGPUS</t>
         </is>
       </c>
       <c r="H24" t="inlineStr"/>
@@ -1585,17 +1585,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-02-23T14:36:04Z</t>
+          <t>2026-06-08T12:24:26Z</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>['ftniigatauniv:oai:niigata-u.repo.nii.ac.jp:00006179']</t>
+          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00025085']</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>['demo', 'socio']</t>
+          <t>['museo']</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -1609,7 +1609,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>__4hQrT1f8FDe4OtrtQJSDK</t>
+          <t>__4KN7H5ulJXhqUvCG7ZrPJ</t>
         </is>
       </c>
       <c r="H25" t="inlineStr"/>
@@ -1633,17 +1633,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-08-14T11:54:29Z</t>
+          <t>2026-02-23T14:36:04Z</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00039136']</t>
+          <t>['ftniigatauniv:oai:niigata-u.repo.nii.ac.jp:00006179']</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>['psy', 'lang']</t>
+          <t>['demo', 'socio']</t>
         </is>
       </c>
       <c r="D26" t="n">
@@ -1657,7 +1657,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>__4eIpzAs05B4ZRv-5WGPUS</t>
+          <t>__4hQrT1f8FDe4OtrtQJSDK</t>
         </is>
       </c>
       <c r="H26" t="inlineStr"/>
@@ -1681,17 +1681,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-06-06T02:58:45Z</t>
+          <t>2026-07-31T03:29:31Z</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00039179']</t>
+          <t>['ftniigatauniv:oai:niigata-u.repo.nii.ac.jp:00002963']</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>['lang']</t>
+          <t>['phil', 'scipo']</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -1705,7 +1705,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>__59RnpZxfku6b3ydsd2b9k</t>
+          <t>__4lDRom4gaaw1FTIom5IUp</t>
         </is>
       </c>
       <c r="H27" t="inlineStr"/>
@@ -1729,17 +1729,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-07-31T03:29:31Z</t>
+          <t>2026-06-06T02:58:45Z</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>['ftniigatauniv:oai:niigata-u.repo.nii.ac.jp:00002963']</t>
+          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00039179']</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>['phil', 'scipo']</t>
+          <t>['lang']</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -1753,7 +1753,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>__4lDRom4gaaw1FTIom5IUp</t>
+          <t>__59RnpZxfku6b3ydsd2b9k</t>
         </is>
       </c>
       <c r="H28" t="inlineStr"/>
@@ -1777,17 +1777,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-02-20T08:04:15Z</t>
+          <t>2026-08-14T11:52:54Z</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>['ftniigatauniv:oai:niigata-u.repo.nii.ac.jp:00001726']</t>
+          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00027456']</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>['info', 'stat']</t>
+          <t>['lang', 'litt']</t>
         </is>
       </c>
       <c r="D29" t="n">
@@ -1801,7 +1801,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>__5y4ls4xd7qwyrCEC7bS7V</t>
+          <t>__65dd7Tb00ujcdzdslmcEh</t>
         </is>
       </c>
       <c r="H29" t="inlineStr"/>
@@ -1825,17 +1825,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-08-14T11:52:54Z</t>
+          <t>2026-07-17T15:59:34Z</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00027456']</t>
+          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00017062']</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>['lang', 'litt']</t>
+          <t>['droit', 'hist']</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -1849,7 +1849,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>__65dd7Tb00ujcdzdslmcEh</t>
+          <t>__6yIH-mPB4rmIpeYYAsJMV</t>
         </is>
       </c>
       <c r="H30" t="inlineStr"/>
@@ -1873,17 +1873,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-07-17T15:59:34Z</t>
+          <t>2026-08-13T14:25:51Z</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00017062']</t>
+          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00027332']</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>['droit', 'hist']</t>
+          <t>['hist', 'socio']</t>
         </is>
       </c>
       <c r="D31" t="n">
@@ -1897,7 +1897,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>__6yIH-mPB4rmIpeYYAsJMV</t>
+          <t>__722aVCcrfxx0yzVebTYZp</t>
         </is>
       </c>
       <c r="H31" t="inlineStr"/>
@@ -1921,17 +1921,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-08-13T14:25:51Z</t>
+          <t>2026-02-20T08:04:15Z</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00027332']</t>
+          <t>['ftniigatauniv:oai:niigata-u.repo.nii.ac.jp:00001726']</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>['hist', 'socio']</t>
+          <t>['info', 'stat']</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -1945,7 +1945,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>__722aVCcrfxx0yzVebTYZp</t>
+          <t>__5y4ls4xd7qwyrCEC7bS7V</t>
         </is>
       </c>
       <c r="H32" t="inlineStr"/>
@@ -2209,17 +2209,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-07-13T10:19:47Z</t>
+          <t>2026-08-08T17:09:27Z</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00031667']</t>
+          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00027113']</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>['hist', 'droit']</t>
+          <t>['scipo', 'hisphilso']</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -2233,7 +2233,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>__9uiaL2Kr6Uuw0yf_D42gg</t>
+          <t>__A2PObfvhgd1RDg_NvM_A5</t>
         </is>
       </c>
       <c r="H38" t="inlineStr"/>
@@ -2305,17 +2305,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-08-08T17:09:27Z</t>
+          <t>2026-08-08T17:09:30Z</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00027113']</t>
+          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00031502']</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>['scipo', 'hisphilso']</t>
+          <t>['scipo', 'edu']</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -2329,7 +2329,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>__A2PObfvhgd1RDg_NvM_A5</t>
+          <t>__AqJW4n8fEFgGBusAOhOaM</t>
         </is>
       </c>
       <c r="H40" t="inlineStr"/>
@@ -2353,17 +2353,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-08-14T13:21:00Z</t>
+          <t>2026-07-13T10:19:47Z</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00031059']</t>
+          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00031667']</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>['psy', 'edu']</t>
+          <t>['hist', 'droit']</t>
         </is>
       </c>
       <c r="D41" t="n">
@@ -2377,7 +2377,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>__AfBBvrYreueEw-popoXhG</t>
+          <t>__9uiaL2Kr6Uuw0yf_D42gg</t>
         </is>
       </c>
       <c r="H41" t="inlineStr"/>
@@ -2401,17 +2401,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-08-08T17:09:30Z</t>
+          <t>2026-08-14T13:21:00Z</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00031502']</t>
+          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00031059']</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>['scipo', 'edu']</t>
+          <t>['psy', 'edu']</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -2425,7 +2425,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>__AqJW4n8fEFgGBusAOhOaM</t>
+          <t>__AfBBvrYreueEw-popoXhG</t>
         </is>
       </c>
       <c r="H42" t="inlineStr"/>
@@ -2689,17 +2689,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-08-14T11:53:07Z</t>
+          <t>2026-03-10T12:38:36Z</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00039194']</t>
+          <t>['ftniigatauniv:oai:niigata-u.repo.nii.ac.jp:00001588']</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>['lang', 'phil']</t>
+          <t>['envir']</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -2713,7 +2713,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>__D2UfFsdGPlI0AB-DGqAoq</t>
+          <t>__DhAO02eKMaJ9ZK2imFJqx</t>
         </is>
       </c>
       <c r="H48" t="inlineStr"/>
@@ -2737,17 +2737,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-08-13T05:07:19Z</t>
+          <t>2026-08-14T13:21:00Z</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00029742']</t>
+          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00031059']</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>['genre', 'socio']</t>
+          <t>['psy', 'edu']</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -2761,7 +2761,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>__Dp5Fssm0mw7OOLf5E7Ryo</t>
+          <t>__DnXXLW1m6dfh9rHD7mIu4</t>
         </is>
       </c>
       <c r="H49" t="inlineStr"/>
@@ -2785,17 +2785,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-03-10T12:38:36Z</t>
+          <t>2026-08-13T05:07:19Z</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>['ftniigatauniv:oai:niigata-u.repo.nii.ac.jp:00001588']</t>
+          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00029742']</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>['envir']</t>
+          <t>['genre', 'socio']</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -2809,7 +2809,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>__DhAO02eKMaJ9ZK2imFJqx</t>
+          <t>__Dp5Fssm0mw7OOLf5E7Ryo</t>
         </is>
       </c>
       <c r="H50" t="inlineStr"/>
@@ -2833,17 +2833,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-08-14T13:21:00Z</t>
+          <t>2026-08-18T07:01:25Z</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00031059']</t>
+          <t>['ftniigatauniv:oai:niigata-u.repo.nii.ac.jp:00002865', 'ftniigatauniv:oai:niigata-u.repo.nii.ac.jp:00030989']</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>['psy', 'edu']</t>
+          <t>['edu', 'lang', 'litt', 'phil', 'hisphilso']</t>
         </is>
       </c>
       <c r="D51" t="n">
@@ -2857,12 +2857,12 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>__DnXXLW1m6dfh9rHD7mIu4</t>
+          <t>__CbwQdx-gEWFktXcVYb8ME</t>
         </is>
       </c>
       <c r="H51" t="inlineStr"/>
       <c r="I51" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J51" t="b">
         <v>0</v>
@@ -2881,17 +2881,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-08-18T07:01:25Z</t>
+          <t>2026-08-14T11:53:07Z</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>['ftniigatauniv:oai:niigata-u.repo.nii.ac.jp:00002865', 'ftniigatauniv:oai:niigata-u.repo.nii.ac.jp:00030989']</t>
+          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00039194']</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>['edu', 'lang', 'litt', 'phil', 'hisphilso']</t>
+          <t>['lang', 'phil']</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -2905,12 +2905,12 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>__CbwQdx-gEWFktXcVYb8ME</t>
+          <t>__D2UfFsdGPlI0AB-DGqAoq</t>
         </is>
       </c>
       <c r="H52" t="inlineStr"/>
       <c r="I52" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J52" t="b">
         <v>0</v>
@@ -2929,17 +2929,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-08-14T12:01:40Z</t>
+          <t>2026-02-23T14:36:04Z</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00000402']</t>
+          <t>['ftniigatauniv:oai:niigata-u.repo.nii.ac.jp:00006179']</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>['lang', 'litt']</t>
+          <t>['demo', 'socio']</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -2953,7 +2953,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>__EJSrO8lPe5qaCdq3DysOG</t>
+          <t>__Dxuo_uNaUGg3mumbQFchm</t>
         </is>
       </c>
       <c r="H53" t="inlineStr"/>
@@ -3025,17 +3025,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-02-23T14:36:04Z</t>
+          <t>2026-08-14T12:01:40Z</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>['ftniigatauniv:oai:niigata-u.repo.nii.ac.jp:00006179']</t>
+          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00000402']</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>['demo', 'socio']</t>
+          <t>['lang', 'litt']</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -3049,7 +3049,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>__Dxuo_uNaUGg3mumbQFchm</t>
+          <t>__EJSrO8lPe5qaCdq3DysOG</t>
         </is>
       </c>
       <c r="H55" t="inlineStr"/>
@@ -3217,17 +3217,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-07-09T19:15:26Z</t>
+          <t>2026-08-08T16:49:51Z</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>['ftniigatauniv:oai:niigata-u.repo.nii.ac.jp:00026817']</t>
+          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00025114']</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>['genre', 'demo']</t>
+          <t>['phil', 'hisphilso']</t>
         </is>
       </c>
       <c r="D59" t="n">
@@ -3241,7 +3241,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>__FJyKuEEQXm-obCqakt7Db</t>
+          <t>__EskvkYA0LYjn7dcQKSB0I</t>
         </is>
       </c>
       <c r="H59" t="inlineStr"/>
@@ -3265,17 +3265,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-08-08T16:49:51Z</t>
+          <t>2026-07-09T19:15:26Z</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00025114']</t>
+          <t>['ftniigatauniv:oai:niigata-u.repo.nii.ac.jp:00026817']</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>['phil', 'hisphilso']</t>
+          <t>['genre', 'demo']</t>
         </is>
       </c>
       <c r="D60" t="n">
@@ -3289,7 +3289,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>__EskvkYA0LYjn7dcQKSB0I</t>
+          <t>__FJyKuEEQXm-obCqakt7Db</t>
         </is>
       </c>
       <c r="H60" t="inlineStr"/>
@@ -3409,17 +3409,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-08-08T17:09:32Z</t>
+          <t>2026-08-14T11:52:59Z</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00031717']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>['scipo', 'socio']</t>
+          <t>['lang', 'litt']</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -3433,12 +3433,12 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>__GeJ0lOVILlQKFGngrsGqa</t>
+          <t>__HLjlO4VJyjm1jh6y4hlYX</t>
         </is>
       </c>
       <c r="H63" t="inlineStr"/>
       <c r="I63" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J63" t="b">
         <v>0</v>
@@ -3457,17 +3457,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-08-08T12:37:17Z</t>
+          <t>2026-08-08T17:09:32Z</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>['ftunivromairis:oai:iris.uniroma1.it:11573_1183823', 'ftchacadscienegi:oai:ir.xjlas.org:365004_10838']</t>
+          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00031717']</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>['psy', 'socio', 'demo', 'eco']</t>
+          <t>['scipo', 'socio']</t>
         </is>
       </c>
       <c r="D64" t="n">
@@ -3481,12 +3481,12 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>__DpaWUjHZQMo7B_9GMMD1x</t>
+          <t>__GeJ0lOVILlQKFGngrsGqa</t>
         </is>
       </c>
       <c r="H64" t="inlineStr"/>
       <c r="I64" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J64" t="b">
         <v>0</v>
@@ -3505,17 +3505,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-07-31T03:29:34Z</t>
+          <t>2026-08-08T12:37:17Z</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>['ftniigatauniv:oai:niigata-u.repo.nii.ac.jp:00007367']</t>
+          <t>['ftunivromairis:oai:iris.uniroma1.it:11573_1183823', 'ftchacadscienegi:oai:ir.xjlas.org:365004_10838']</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>['scipo', 'hist']</t>
+          <t>['psy', 'socio', 'demo', 'eco']</t>
         </is>
       </c>
       <c r="D65" t="n">
@@ -3529,12 +3529,12 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>__GulDaDah1yGGWLg-Cl8Yc</t>
+          <t>__DpaWUjHZQMo7B_9GMMD1x</t>
         </is>
       </c>
       <c r="H65" t="inlineStr"/>
       <c r="I65" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J65" t="b">
         <v>0</v>
@@ -3553,17 +3553,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-08-14T11:52:59Z</t>
+          <t>2026-07-31T03:29:34Z</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['ftniigatauniv:oai:niigata-u.repo.nii.ac.jp:00007367']</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>['lang', 'litt']</t>
+          <t>['scipo', 'hist']</t>
         </is>
       </c>
       <c r="D66" t="n">
@@ -3577,12 +3577,12 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>__HLjlO4VJyjm1jh6y4hlYX</t>
+          <t>__GulDaDah1yGGWLg-Cl8Yc</t>
         </is>
       </c>
       <c r="H66" t="inlineStr"/>
       <c r="I66" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J66" t="b">
         <v>0</v>
@@ -3649,17 +3649,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-08-13T22:45:58Z</t>
+          <t>2026-07-13T10:19:41Z</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>['ftniigatauniv:oai:niigata-u.repo.nii.ac.jp:00007987']</t>
+          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00031517']</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>['lang', 'demo']</t>
+          <t>['scipo', 'hist']</t>
         </is>
       </c>
       <c r="D68" t="n">
@@ -3673,7 +3673,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>__Ic3qvlSt2gMH81OUwECWq</t>
+          <t>__HORV6k_x5UWJWiUb82kJc</t>
         </is>
       </c>
       <c r="H68" t="inlineStr"/>
@@ -3697,17 +3697,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-07-13T10:19:41Z</t>
+          <t>2026-08-13T22:45:58Z</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00031517']</t>
+          <t>['ftniigatauniv:oai:niigata-u.repo.nii.ac.jp:00007987']</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>['scipo', 'hist']</t>
+          <t>['lang', 'demo']</t>
         </is>
       </c>
       <c r="D69" t="n">
@@ -3721,7 +3721,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>__HORV6k_x5UWJWiUb82kJc</t>
+          <t>__Ic3qvlSt2gMH81OUwECWq</t>
         </is>
       </c>
       <c r="H69" t="inlineStr"/>
@@ -3745,17 +3745,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-08-14T13:09:36Z</t>
+          <t>2026-08-08T17:09:22Z</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00029930']</t>
+          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00016946']</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>['psy', 'lang']</t>
+          <t>['scipo', 'socio']</t>
         </is>
       </c>
       <c r="D70" t="n">
@@ -3769,7 +3769,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>__IhMd4k0GK6q60sMEFCtNR</t>
+          <t>__IiVpgWALlwDqvM5_urj6S</t>
         </is>
       </c>
       <c r="H70" t="inlineStr"/>
@@ -3793,17 +3793,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-08-08T17:09:22Z</t>
+          <t>2026-08-14T13:09:36Z</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00016946']</t>
+          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00029930']</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>['scipo', 'socio']</t>
+          <t>['psy', 'lang']</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -3817,7 +3817,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>__IiVpgWALlwDqvM5_urj6S</t>
+          <t>__IhMd4k0GK6q60sMEFCtNR</t>
         </is>
       </c>
       <c r="H71" t="inlineStr"/>
@@ -3889,17 +3889,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-08-08T17:09:25Z</t>
+          <t>2026-07-13T14:57:17Z</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00017707']</t>
+          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00031323']</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>['hist', 'socio']</t>
+          <t>['socio', 'litt']</t>
         </is>
       </c>
       <c r="D73" t="n">
@@ -3913,7 +3913,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>__JUPhcMA-nBLk8duDUzo4g</t>
+          <t>__JsUS-TJQq2MeqQOXz2j3e</t>
         </is>
       </c>
       <c r="H73" t="inlineStr"/>
@@ -3937,17 +3937,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-07-13T14:57:17Z</t>
+          <t>2026-08-08T17:09:25Z</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00031323']</t>
+          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00017707']</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>['socio', 'litt']</t>
+          <t>['hist', 'socio']</t>
         </is>
       </c>
       <c r="D74" t="n">
@@ -3961,7 +3961,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>__JsUS-TJQq2MeqQOXz2j3e</t>
+          <t>__JUPhcMA-nBLk8duDUzo4g</t>
         </is>
       </c>
       <c r="H74" t="inlineStr"/>
@@ -3985,17 +3985,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-06-07T23:57:06Z</t>
+          <t>2026-08-14T13:09:36Z</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00030534']</t>
+          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00029930']</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>['relig', 'hisphilso']</t>
+          <t>['psy', 'lang']</t>
         </is>
       </c>
       <c r="D75" t="n">
@@ -4009,7 +4009,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>__Kn_alAO1yru5IfyMnNh99</t>
+          <t>__K8U1IzoCR_pny3OPWLsv5</t>
         </is>
       </c>
       <c r="H75" t="inlineStr"/>
@@ -4033,17 +4033,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-08-14T13:09:36Z</t>
+          <t>2026-06-07T23:57:06Z</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00029930']</t>
+          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00030534']</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>['psy', 'lang']</t>
+          <t>['relig', 'hisphilso']</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -4057,7 +4057,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>__K8U1IzoCR_pny3OPWLsv5</t>
+          <t>__Kn_alAO1yru5IfyMnNh99</t>
         </is>
       </c>
       <c r="H76" t="inlineStr"/>
@@ -4081,17 +4081,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-02-20T08:04:15Z</t>
+          <t>2026-06-07T11:02:07Z</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>['ftniigatauniv:oai:niigata-u.repo.nii.ac.jp:00001726']</t>
+          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00027479']</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>['info', 'stat']</t>
+          <t>['lang', 'litt']</t>
         </is>
       </c>
       <c r="D77" t="n">
@@ -4105,7 +4105,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>__L00MemwgttgXlcetVWQz8</t>
+          <t>__Kx2k4Pin1eTDdzQsDycZN</t>
         </is>
       </c>
       <c r="H77" t="inlineStr"/>
@@ -4129,17 +4129,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-08-14T11:53:44Z</t>
+          <t>2026-02-20T08:04:15Z</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00027549']</t>
+          <t>['ftniigatauniv:oai:niigata-u.repo.nii.ac.jp:00001726']</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>['lang', 'litt']</t>
+          <t>['info', 'stat']</t>
         </is>
       </c>
       <c r="D78" t="n">
@@ -4153,7 +4153,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>__LBtqT5kr37uJ7wjutlun5</t>
+          <t>__L00MemwgttgXlcetVWQz8</t>
         </is>
       </c>
       <c r="H78" t="inlineStr"/>
@@ -4177,12 +4177,12 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-06-07T11:02:07Z</t>
+          <t>2026-08-14T11:53:44Z</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00027479']</t>
+          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00027549']</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -4201,7 +4201,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>__Kx2k4Pin1eTDdzQsDycZN</t>
+          <t>__LBtqT5kr37uJ7wjutlun5</t>
         </is>
       </c>
       <c r="H79" t="inlineStr"/>
@@ -4321,17 +4321,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-08-10T07:13:51Z</t>
+          <t>2026-07-13T10:19:37Z</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>['ftniigatauniv:oai:niigata-u.repo.nii.ac.jp:00028528']</t>
+          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00025143']</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>['socio', 'psy']</t>
+          <t>['lang', 'hisphilso']</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -4345,7 +4345,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>__MULZnpMXeBHFci0iVcCK6</t>
+          <t>__LlIeHSXS7_3jX0-67Odha</t>
         </is>
       </c>
       <c r="H82" t="inlineStr"/>
@@ -4369,17 +4369,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-07-13T10:19:37Z</t>
+          <t>2026-08-13T22:46:15Z</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00025143']</t>
+          <t>['ftniigatauniv:oai:niigata-u.repo.nii.ac.jp:00027122']</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>['lang', 'hisphilso']</t>
+          <t>['lang', 'litt']</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -4393,7 +4393,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>__LlIeHSXS7_3jX0-67Odha</t>
+          <t>__MEvh03EPyCTDz8xEecDnx</t>
         </is>
       </c>
       <c r="H83" t="inlineStr"/>
@@ -4417,17 +4417,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-08-13T22:46:15Z</t>
+          <t>2026-08-10T07:13:51Z</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>['ftniigatauniv:oai:niigata-u.repo.nii.ac.jp:00027122']</t>
+          <t>['ftniigatauniv:oai:niigata-u.repo.nii.ac.jp:00028528']</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>['lang', 'litt']</t>
+          <t>['socio', 'psy']</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -4441,7 +4441,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>__MEvh03EPyCTDz8xEecDnx</t>
+          <t>__MULZnpMXeBHFci0iVcCK6</t>
         </is>
       </c>
       <c r="H84" t="inlineStr"/>
@@ -4561,17 +4561,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-08-14T12:01:40Z</t>
+          <t>2026-08-08T17:09:23Z</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00000402']</t>
+          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00017058']</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>['lang', 'litt']</t>
+          <t>['scipo', 'hist']</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -4585,7 +4585,7 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>__OT_5CrYbEI4IxQkuGBI9x</t>
+          <t>__OHTo8WdCa2SUVHNshP2d7</t>
         </is>
       </c>
       <c r="H87" t="inlineStr"/>
@@ -4609,17 +4609,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-08-13T04:59:15Z</t>
+          <t>2026-08-14T12:01:40Z</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00031051']</t>
+          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00000402']</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>['hisphilso', 'socio']</t>
+          <t>['lang', 'litt']</t>
         </is>
       </c>
       <c r="D88" t="n">
@@ -4633,7 +4633,7 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>__Oar71J7VzZOSGkXrIjV9g</t>
+          <t>__OT_5CrYbEI4IxQkuGBI9x</t>
         </is>
       </c>
       <c r="H88" t="inlineStr"/>
@@ -4705,17 +4705,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-07-13T12:24:54Z</t>
+          <t>2026-08-13T04:59:09Z</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00031087']</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>['anthro-se', 'hisphilso']</t>
+          <t>['archeo', 'hist']</t>
         </is>
       </c>
       <c r="D90" t="n">
@@ -4729,12 +4729,12 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>__Ov0QH6Msk9Rx9OHgWOqad</t>
+          <t>__P92IJiRexY6MZa_XDO4q9</t>
         </is>
       </c>
       <c r="H90" t="inlineStr"/>
       <c r="I90" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J90" t="b">
         <v>0</v>
@@ -4753,17 +4753,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-08-13T04:59:09Z</t>
+          <t>2026-08-13T04:59:15Z</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00031051']</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>['archeo', 'hist']</t>
+          <t>['hisphilso', 'socio']</t>
         </is>
       </c>
       <c r="D91" t="n">
@@ -4777,12 +4777,12 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>__P92IJiRexY6MZa_XDO4q9</t>
+          <t>__Oar71J7VzZOSGkXrIjV9g</t>
         </is>
       </c>
       <c r="H91" t="inlineStr"/>
       <c r="I91" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J91" t="b">
         <v>0</v>
@@ -4801,17 +4801,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-08-08T17:09:23Z</t>
+          <t>2026-07-17T15:59:21Z</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00017058']</t>
+          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00031635']</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>['scipo', 'hist']</t>
+          <t>['droit', 'socio']</t>
         </is>
       </c>
       <c r="D92" t="n">
@@ -4825,7 +4825,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>__OHTo8WdCa2SUVHNshP2d7</t>
+          <t>__P2Nz3NiYJNvlDhXWpPcP8</t>
         </is>
       </c>
       <c r="H92" t="inlineStr"/>
@@ -4897,17 +4897,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-08-10T07:13:50Z</t>
+          <t>2026-07-13T12:24:54Z</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>['ftniigatauniv:oai:niigata-u.repo.nii.ac.jp:00028528']</t>
+          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00031087']</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>['socio', 'psy']</t>
+          <t>['anthro-se', 'hisphilso']</t>
         </is>
       </c>
       <c r="D94" t="n">
@@ -4921,7 +4921,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>__P9CtP_bkIRKQwUfHRKIgr</t>
+          <t>__Ov0QH6Msk9Rx9OHgWOqad</t>
         </is>
       </c>
       <c r="H94" t="inlineStr"/>
@@ -4945,17 +4945,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-08-07T16:01:47Z</t>
+          <t>2026-08-10T07:13:50Z</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00026859']</t>
+          <t>['ftniigatauniv:oai:niigata-u.repo.nii.ac.jp:00028528']</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>['hist', 'archi']</t>
+          <t>['socio', 'psy']</t>
         </is>
       </c>
       <c r="D95" t="n">
@@ -4969,7 +4969,7 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>__PyEOaoi8CHBdziFLeHRna</t>
+          <t>__P9CtP_bkIRKQwUfHRKIgr</t>
         </is>
       </c>
       <c r="H95" t="inlineStr"/>
@@ -4993,17 +4993,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-08-14T11:52:54Z</t>
+          <t>2026-08-07T16:01:47Z</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00027488']</t>
+          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00026859']</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>['lang', 'phil']</t>
+          <t>['hist', 'archi']</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -5017,7 +5017,7 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>__Q8PhgVa3HWHZSD_Ly4OUE</t>
+          <t>__PyEOaoi8CHBdziFLeHRna</t>
         </is>
       </c>
       <c r="H96" t="inlineStr"/>
@@ -5041,17 +5041,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-07-17T15:59:21Z</t>
+          <t>2026-08-14T11:52:54Z</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00031635']</t>
+          <t>['ftunivtokyo:oai:repository.dl.itc.u-tokyo.ac.jp:00027488']</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>['droit', 'socio']</t>
+          <t>['lang', 'phil']</t>
         </is>
       </c>
       <c r="D97" t="n">
@@ -5065,7 +5065,7 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>__P2Nz3NiYJNvlDhXWpPcP8</t>
+          <t>__Q8PhgVa3HWHZSD_Ly4OUE</t>
         </is>
       </c>
       <c r="H97" t="inlineStr"/>

</xml_diff>